<commit_message>
Added Example script to run.
</commit_message>
<xml_diff>
--- a/statistics/model_statistics/model_statistics.xlsx
+++ b/statistics/model_statistics/model_statistics.xlsx
@@ -1,58 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shaad Hafeez\CODE\HYBRIDMODELS\statistics\model_statistics\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED57C60-ADD2-4CFC-8DA4-0A352765DB55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>Model</t>
-  </si>
-  <si>
-    <t>Rsquared</t>
-  </si>
-  <si>
-    <t>arima</t>
-  </si>
-  <si>
-    <t>MSE</t>
-  </si>
-  <si>
-    <t>MAPE</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -71,21 +46,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -373,36 +407,57 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col width="13.5546875" bestFit="1" customWidth="1" min="1" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Rsquared</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>MSE</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>MAPE</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
-        <v>0.92068381123045506</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>arima</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.9206838112304551</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>arimadiff-mlp</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>6472.88940812202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final Commit to remove unneccessary code
</commit_message>
<xml_diff>
--- a/statistics/model_statistics/model_statistics.xlsx
+++ b/statistics/model_statistics/model_statistics.xlsx
@@ -1,33 +1,79 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shaad Hafeez\CODE\HYBRIDMODELS\statistics\model_statistics\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDABDD2C-00CA-43FC-A596-AABA2CFD951A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Rsquared</t>
+  </si>
+  <si>
+    <t>MAE</t>
+  </si>
+  <si>
+    <t>MSE</t>
+  </si>
+  <si>
+    <t>MAPE</t>
+  </si>
+  <si>
+    <t>Hit Rate</t>
+  </si>
+  <si>
+    <t>VARMAX-LSTM</t>
+  </si>
+  <si>
+    <t>VARMAX-SVR</t>
+  </si>
+  <si>
+    <t>VARMAX-GBR</t>
+  </si>
+  <si>
+    <t>VARMAX-MLP</t>
+  </si>
+  <si>
+    <t>VARMAX-LGBM</t>
+  </si>
+  <si>
+    <t>VARMAX</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,80 +92,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -134,28 +121,28 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="0000FF"/>
@@ -257,6 +244,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
@@ -267,31 +255,27 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="9500"/>
+              <a:shade val="95000"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
@@ -313,7 +297,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -371,7 +355,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="20000"/>
+                <a:shade val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -384,12 +368,13 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
+                <a:shade val="30000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -401,66 +386,196 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="13.5546875" bestFit="1" customWidth="1" min="1" max="2"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Rsquared</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>MSE</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>MAPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>arima</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.9206838112304551</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>arimadiff-mlp</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>6472.88940812202</v>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>0.88535255226678033</v>
+      </c>
+      <c r="C2">
+        <v>3.20212527930744</v>
+      </c>
+      <c r="D2">
+        <v>21.663909925618661</v>
+      </c>
+      <c r="E2">
+        <v>0.12459634881542921</v>
+      </c>
+      <c r="F2">
+        <v>0.49016064257028108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>0.99334446879288618</v>
+      </c>
+      <c r="C3">
+        <v>0.92117230594658839</v>
+      </c>
+      <c r="D3">
+        <v>1.278057382147276</v>
+      </c>
+      <c r="E3">
+        <v>4.396427283605122E-2</v>
+      </c>
+      <c r="F3">
+        <v>0.49203187250996022</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>0.9728404693811834</v>
+      </c>
+      <c r="C4">
+        <v>1.3534857091248631</v>
+      </c>
+      <c r="D4">
+        <v>5.1007604501292398</v>
+      </c>
+      <c r="E4">
+        <v>5.2659866255665287E-2</v>
+      </c>
+      <c r="F4">
+        <v>0.4892430278884462</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>0.98779866747211087</v>
+      </c>
+      <c r="C5">
+        <v>0.70318525357248418</v>
+      </c>
+      <c r="D5">
+        <v>2.2409065088028011</v>
+      </c>
+      <c r="E5">
+        <v>2.9644494853142168E-2</v>
+      </c>
+      <c r="F5">
+        <v>0.50816733067729081</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>0.90058556702248815</v>
+      </c>
+      <c r="C6">
+        <v>3.0092530614862611</v>
+      </c>
+      <c r="D6">
+        <v>18.820608748452251</v>
+      </c>
+      <c r="E6">
+        <v>0.11440609735807709</v>
+      </c>
+      <c r="F6">
+        <v>0.49442231075697213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>0.8926972451757802</v>
+      </c>
+      <c r="C7">
+        <v>3.070295033790011</v>
+      </c>
+      <c r="D7">
+        <v>20.301538374180719</v>
+      </c>
+      <c r="E7">
+        <v>0.1159622966111177</v>
+      </c>
+      <c r="F7">
+        <v>0.49442231075697213</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>